<commit_message>
adjusted parametrization for stabilized Nm balance
</commit_message>
<xml_diff>
--- a/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
+++ b/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sshfs\torisuten@192.168.12.9\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E1F9BE-3A28-4B2F-84E7-ABD8A18F2AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0F3162-BBD0-4589-865F-69823563E650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -3426,7 +3426,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="J2" s="9">
-        <v>1E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>179</v>
@@ -3767,10 +3767,10 @@
         <v>-10000000</v>
       </c>
       <c r="J8" s="9">
-        <v>-10000</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>179</v>
+        <v>-100</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="L8" s="4" t="s">
         <v>187</v>
@@ -3885,7 +3885,7 @@
         <v>2.0663913021965896E-9</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="L10" s="4" t="s">
         <v>188</v>

</xml_diff>

<commit_message>
added new axial N transport model along with previous one, based on the hypothesis of radial water uptake restricting / dilluting incomming fluxes progress (previous segments in the moving column and radial fluxes, without forgetting advection but which seems minor)
</commit_message>
<xml_diff>
--- a/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
+++ b/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sshfs\torisuten@192.168.12.9\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0F3162-BBD0-4589-865F-69823563E650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9583E9-5E0C-4A24-B548-9A3CAF0473D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3429,7 +3429,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>188</v>
@@ -3655,8 +3655,8 @@
       <c r="J6" s="9">
         <v>4.6999999999999999E-4</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>179</v>
+      <c r="K6" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>187</v>

</xml_diff>

<commit_message>
equal contribution of active and passive hexose production from phloem for better stability of hexose allocation
</commit_message>
<xml_diff>
--- a/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
+++ b/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sshfs\torisuten@192.168.12.9\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9583E9-5E0C-4A24-B548-9A3CAF0473D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC1FD61-6C65-4767-93BF-82204EBF433D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -3325,21 +3325,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil1"/>
   <dimension ref="A1:R30"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="32.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" customWidth="1"/>
     <col min="5" max="6" width="17" customWidth="1"/>
-    <col min="7" max="8" width="19.54296875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="15.81640625" style="1" customWidth="1"/>
-    <col min="10" max="16" width="15.1796875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="19.7265625" customWidth="1"/>
-    <col min="18" max="18" width="20.7265625" customWidth="1"/>
+    <col min="7" max="8" width="19.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="1" customWidth="1"/>
+    <col min="10" max="16" width="15.140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="19.7109375" customWidth="1"/>
+    <col min="18" max="18" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>290</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>275</v>
       </c>
@@ -3434,8 +3434,8 @@
       <c r="L2" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="M2" s="16" t="s">
-        <v>175</v>
+      <c r="M2" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="N2" s="9" t="s">
         <v>179</v>
@@ -3453,7 +3453,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>291</v>
       </c>
@@ -3495,8 +3495,8 @@
       <c r="L3" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>175</v>
+      <c r="M3" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="N3" s="9" t="s">
         <v>179</v>
@@ -3514,7 +3514,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>190</v>
       </c>
@@ -3549,14 +3549,14 @@
       <c r="L4" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="M4" s="15" t="s">
-        <v>175</v>
+      <c r="M4" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="N4" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="O4" s="4" t="s">
-        <v>179</v>
+      <c r="O4" s="15" t="s">
+        <v>175</v>
       </c>
       <c r="P4" s="4" t="s">
         <v>179</v>
@@ -3568,7 +3568,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>190</v>
       </c>
@@ -3626,7 +3626,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>195</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>239</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>326</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>240</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>248</v>
       </c>
@@ -3890,8 +3890,8 @@
       <c r="L10" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="M10" s="15" t="s">
-        <v>175</v>
+      <c r="M10" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="N10" s="4" t="s">
         <v>179</v>
@@ -3911,7 +3911,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>293</v>
       </c>
@@ -3949,8 +3949,8 @@
       <c r="L11" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="M11" s="15" t="s">
-        <v>175</v>
+      <c r="M11" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="N11" s="4" t="s">
         <v>179</v>
@@ -3970,7 +3970,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="16:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="16:16" x14ac:dyDescent="0.25">
       <c r="P30" s="10"/>
     </row>
   </sheetData>
@@ -4000,30 +4000,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1409DA-5B3D-4C19-B6DA-5F98667DB196}">
   <sheetPr codeName="Feuil2"/>
   <dimension ref="A1:AC7"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="17.81640625" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
     <col min="6" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="14.26953125" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" customWidth="1"/>
-    <col min="11" max="11" width="23.26953125" customWidth="1"/>
-    <col min="12" max="15" width="19.7265625" customWidth="1"/>
-    <col min="16" max="16" width="21.7265625" customWidth="1"/>
-    <col min="17" max="17" width="17.1796875" customWidth="1"/>
-    <col min="18" max="18" width="18.453125" customWidth="1"/>
-    <col min="19" max="19" width="21.1796875" customWidth="1"/>
-    <col min="20" max="20" width="14.26953125" customWidth="1"/>
-    <col min="22" max="25" width="16.81640625" customWidth="1"/>
-    <col min="26" max="26" width="43.453125" customWidth="1"/>
-    <col min="27" max="29" width="21.1796875" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="23.28515625" customWidth="1"/>
+    <col min="12" max="15" width="19.7109375" customWidth="1"/>
+    <col min="16" max="16" width="21.7109375" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" customWidth="1"/>
+    <col min="18" max="18" width="18.42578125" customWidth="1"/>
+    <col min="19" max="19" width="21.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.28515625" customWidth="1"/>
+    <col min="22" max="25" width="16.85546875" customWidth="1"/>
+    <col min="26" max="26" width="43.42578125" customWidth="1"/>
+    <col min="27" max="29" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>199</v>
       </c>
@@ -4112,7 +4112,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>190</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="75.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:29" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>248</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>293</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>248</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>246</v>
       </c>
@@ -4607,7 +4607,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>180</v>
       </c>
@@ -4635,17 +4635,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95EE4405-B4C3-46B7-B8B8-F3A59345C99B}">
   <sheetPr codeName="Feuil3"/>
   <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" customWidth="1"/>
-    <col min="3" max="3" width="35.81640625" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" customWidth="1"/>
-    <col min="5" max="5" width="25.7265625" customWidth="1"/>
-    <col min="6" max="6" width="23.54296875" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>261</v>
       </c>
@@ -4686,7 +4686,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>3.5251481666477781E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>4.0225758996114214E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
@@ -4814,7 +4814,7 @@
         <v>4.5901948239304748E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>6</v>
       </c>
@@ -4854,7 +4854,7 @@
         <v>4.9033687479195865E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>35</v>
       </c>
@@ -4893,127 +4893,127 @@
         <v>3.3245601361544835E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -5029,13 +5029,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20A3C74-7DFC-4CEB-A83D-886DEB62D87A}">
   <sheetPr codeName="Feuil4"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.26953125" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>274</v>
       </c>
@@ -5055,7 +5055,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>278</v>
       </c>
@@ -5085,13 +5085,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Feuil5"/>
   <dimension ref="A1:C169"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.7265625" customWidth="1"/>
-    <col min="3" max="3" width="49.54296875" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>167</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -5114,7 +5114,7 @@
         <v>pi</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5126,7 +5126,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -5150,7 +5150,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -5174,7 +5174,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -5186,7 +5186,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -5198,7 +5198,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -5210,7 +5210,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -5222,7 +5222,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -5246,7 +5246,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>86</v>
       </c>
@@ -5258,7 +5258,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -5282,7 +5282,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -5294,7 +5294,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -5306,7 +5306,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -5318,7 +5318,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -5330,7 +5330,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -5366,7 +5366,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -5390,7 +5390,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -5402,7 +5402,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -5414,7 +5414,7 @@
         <v>root_growth_T_ref</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>root_growth_A</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -5438,7 +5438,7 @@
         <v>root_growth_B</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>95</v>
       </c>
@@ -5450,7 +5450,7 @@
         <v>root_growth_C</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>96</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>97</v>
       </c>
@@ -5474,7 +5474,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>98</v>
       </c>
@@ -5486,7 +5486,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>99</v>
       </c>
@@ -5498,7 +5498,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>100</v>
       </c>
@@ -5510,7 +5510,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>61</v>
       </c>
@@ -5522,7 +5522,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -5534,7 +5534,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>101</v>
       </c>
@@ -5546,7 +5546,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>102</v>
       </c>
@@ -5558,7 +5558,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>103</v>
       </c>
@@ -5570,7 +5570,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -5582,7 +5582,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>76</v>
       </c>
@@ -5594,7 +5594,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>105</v>
       </c>
@@ -5606,7 +5606,7 @@
         <v>expected_C_sucrose_root</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>106</v>
       </c>
@@ -5618,7 +5618,7 @@
         <v>expected_C_hexose_root</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>107</v>
       </c>
@@ -5630,7 +5630,7 @@
         <v>expected_C_hexose_soil</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>108</v>
       </c>
@@ -5642,7 +5642,7 @@
         <v>expected_C_hexose_reserve</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>65</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>77</v>
       </c>
@@ -5666,7 +5666,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>surfacic_unloading_rate_reference</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>110</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>surfacic_unloading_rate_primordium</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -5702,7 +5702,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>111</v>
       </c>
@@ -5714,7 +5714,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>112</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>113</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>114</v>
       </c>
@@ -5750,7 +5750,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -5762,7 +5762,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>115</v>
       </c>
@@ -5774,7 +5774,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>116</v>
       </c>
@@ -5786,7 +5786,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>117</v>
       </c>
@@ -5798,7 +5798,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>118</v>
       </c>
@@ -5810,7 +5810,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -5834,7 +5834,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -5846,7 +5846,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -5858,7 +5858,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>56</v>
       </c>
@@ -5870,7 +5870,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>58</v>
       </c>
@@ -5882,7 +5882,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -5894,7 +5894,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>119</v>
       </c>
@@ -5906,7 +5906,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>120</v>
       </c>
@@ -5918,7 +5918,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>121</v>
       </c>
@@ -5930,7 +5930,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>122</v>
       </c>
@@ -5942,7 +5942,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -5954,7 +5954,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -5966,7 +5966,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>123</v>
       </c>
@@ -5978,7 +5978,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>124</v>
       </c>
@@ -5990,7 +5990,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>125</v>
       </c>
@@ -6002,7 +6002,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>126</v>
       </c>
@@ -6014,7 +6014,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>74</v>
       </c>
@@ -6026,7 +6026,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>127</v>
       </c>
@@ -6038,7 +6038,7 @@
         <v>expected_exudation_efflux</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>128</v>
       </c>
@@ -6062,7 +6062,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>129</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>130</v>
       </c>
@@ -6086,7 +6086,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>131</v>
       </c>
@@ -6098,7 +6098,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -6110,7 +6110,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>80</v>
       </c>
@@ -6122,7 +6122,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>132</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>133</v>
       </c>
@@ -6146,7 +6146,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>134</v>
       </c>
@@ -6158,7 +6158,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>135</v>
       </c>
@@ -6170,7 +6170,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>136</v>
       </c>
@@ -6194,7 +6194,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>137</v>
       </c>
@@ -6206,7 +6206,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>138</v>
       </c>
@@ -6218,7 +6218,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>139</v>
       </c>
@@ -6230,7 +6230,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>140</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>141</v>
       </c>
@@ -6254,7 +6254,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>142</v>
       </c>
@@ -6266,7 +6266,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>143</v>
       </c>
@@ -6278,7 +6278,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>144</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>145</v>
       </c>
@@ -6302,7 +6302,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>146</v>
       </c>
@@ -6314,7 +6314,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>147</v>
       </c>
@@ -6326,7 +6326,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>148</v>
       </c>
@@ -6338,7 +6338,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>149</v>
       </c>
@@ -6350,7 +6350,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>150</v>
       </c>
@@ -6362,7 +6362,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>151</v>
       </c>
@@ -6374,7 +6374,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>152</v>
       </c>
@@ -6386,7 +6386,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>153</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>154</v>
       </c>
@@ -6410,7 +6410,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>155</v>
       </c>
@@ -6422,7 +6422,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>156</v>
       </c>
@@ -6434,7 +6434,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>157</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>158</v>
       </c>
@@ -6458,7 +6458,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>159</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>160</v>
       </c>
@@ -6482,7 +6482,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>161</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>162</v>
       </c>
@@ -6506,7 +6506,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>163</v>
       </c>
@@ -6518,7 +6518,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>164</v>
       </c>
@@ -6530,7 +6530,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>165</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>166</v>
       </c>
@@ -6554,7 +6554,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>59</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>62</v>
       </c>
@@ -6578,7 +6578,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>64</v>
       </c>
@@ -6590,7 +6590,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>63</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>82</v>
       </c>
@@ -6614,7 +6614,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>83</v>
       </c>
@@ -6626,7 +6626,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>85</v>
       </c>
@@ -6638,7 +6638,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>84</v>
       </c>
@@ -6650,7 +6650,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>2</v>
       </c>
@@ -6662,7 +6662,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>20</v>
       </c>
@@ -6698,7 +6698,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>0</v>
       </c>
@@ -6710,7 +6710,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>1</v>
       </c>
@@ -6722,7 +6722,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>6</v>
       </c>
@@ -6734,7 +6734,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>7</v>
       </c>
@@ -6746,7 +6746,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -6758,7 +6758,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -6770,7 +6770,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>10</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>11</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>12</v>
       </c>
@@ -6806,7 +6806,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -6818,7 +6818,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -6830,7 +6830,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>15</v>
       </c>
@@ -6842,7 +6842,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -6854,7 +6854,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>17</v>
       </c>
@@ -6866,7 +6866,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -6878,7 +6878,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>19</v>
       </c>
@@ -6890,7 +6890,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -6902,7 +6902,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>22</v>
       </c>
@@ -6914,7 +6914,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>23</v>
       </c>
@@ -6926,7 +6926,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -6938,7 +6938,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>25</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>27</v>
       </c>
@@ -6974,7 +6974,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>28</v>
       </c>
@@ -6983,7 +6983,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>29</v>
       </c>
@@ -6992,7 +6992,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -7001,7 +7001,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>31</v>
       </c>
@@ -7010,7 +7010,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>33</v>
       </c>
@@ -7028,7 +7028,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -7037,7 +7037,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>35</v>
       </c>
@@ -7046,7 +7046,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>36</v>
       </c>
@@ -7055,7 +7055,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>37</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>38</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>170</v>
       </c>

</xml_diff>

<commit_message>
changed parametrization and inputs
</commit_message>
<xml_diff>
--- a/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
+++ b/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp46580\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEA88A02-AD00-4F05-B431-B70146B79277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828CF325-9EA2-4EB3-97CC-8ABFC52BD208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1073,9 +1073,6 @@
     <t>deficit_AA_phloem</t>
   </si>
   <si>
-    <t>deficit__xylem_Nm</t>
-  </si>
-  <si>
     <t>deficit_xylem_AA</t>
   </si>
   <si>
@@ -1086,6 +1083,9 @@
   </si>
   <si>
     <t>deficit_sucrose_root</t>
+  </si>
+  <si>
+    <t>deficit_xylem_Nm</t>
   </si>
 </sst>
 </file>
@@ -3364,21 +3364,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil1"/>
   <dimension ref="A1:S30"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" customWidth="1"/>
     <col min="5" max="6" width="17" customWidth="1"/>
-    <col min="7" max="8" width="19.5546875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" style="1" customWidth="1"/>
-    <col min="10" max="17" width="15.109375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.6640625" customWidth="1"/>
-    <col min="19" max="19" width="20.6640625" customWidth="1"/>
+    <col min="7" max="8" width="19.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="1" customWidth="1"/>
+    <col min="10" max="17" width="15.140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.7109375" customWidth="1"/>
+    <col min="19" max="19" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>290</v>
       </c>
@@ -3437,7 +3437,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>275</v>
       </c>
@@ -3496,7 +3496,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>291</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>190</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>190</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>195</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>239</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>326</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>240</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>248</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>293</v>
       </c>
@@ -4025,9 +4025,9 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>332</v>
@@ -4082,7 +4082,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>330</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>333</v>
       </c>
@@ -4196,7 +4196,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>334</v>
       </c>
@@ -4253,9 +4253,9 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>332</v>
@@ -4310,9 +4310,9 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>332</v>
@@ -4367,9 +4367,9 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>332</v>
@@ -4424,9 +4424,9 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>332</v>
@@ -4481,7 +4481,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
       <c r="Q30" s="10"/>
     </row>
   </sheetData>
@@ -4535,30 +4535,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1409DA-5B3D-4C19-B6DA-5F98667DB196}">
   <sheetPr codeName="Feuil2"/>
   <dimension ref="A1:AC7"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
     <col min="6" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" customWidth="1"/>
-    <col min="11" max="11" width="23.33203125" customWidth="1"/>
-    <col min="12" max="15" width="19.6640625" customWidth="1"/>
-    <col min="16" max="16" width="21.6640625" customWidth="1"/>
-    <col min="17" max="17" width="17.109375" customWidth="1"/>
-    <col min="18" max="18" width="18.44140625" customWidth="1"/>
-    <col min="19" max="19" width="21.109375" customWidth="1"/>
-    <col min="20" max="20" width="14.33203125" customWidth="1"/>
-    <col min="22" max="25" width="16.88671875" customWidth="1"/>
-    <col min="26" max="26" width="43.44140625" customWidth="1"/>
-    <col min="27" max="29" width="21.109375" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="23.28515625" customWidth="1"/>
+    <col min="12" max="15" width="19.7109375" customWidth="1"/>
+    <col min="16" max="16" width="21.7109375" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" customWidth="1"/>
+    <col min="18" max="18" width="18.42578125" customWidth="1"/>
+    <col min="19" max="19" width="21.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.28515625" customWidth="1"/>
+    <col min="22" max="25" width="16.85546875" customWidth="1"/>
+    <col min="26" max="26" width="43.42578125" customWidth="1"/>
+    <col min="27" max="29" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>199</v>
       </c>
@@ -4647,7 +4647,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>190</v>
       </c>
@@ -4744,7 +4744,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="75.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>248</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>293</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>248</v>
       </c>
@@ -5043,7 +5043,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>246</v>
       </c>
@@ -5142,7 +5142,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>180</v>
       </c>
@@ -5170,17 +5170,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95EE4405-B4C3-46B7-B8B8-F3A59345C99B}">
   <sheetPr codeName="Feuil3"/>
   <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>261</v>
       </c>
@@ -5221,7 +5221,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>3.5251481666477781E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -5309,7 +5309,7 @@
         <v>4.0225758996114214E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>4.5901948239304748E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>6</v>
       </c>
@@ -5389,7 +5389,7 @@
         <v>4.9033687479195865E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>35</v>
       </c>
@@ -5428,127 +5428,127 @@
         <v>3.3245601361544835E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -5564,13 +5564,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20A3C74-7DFC-4CEB-A83D-886DEB62D87A}">
   <sheetPr codeName="Feuil4"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>274</v>
       </c>
@@ -5590,7 +5590,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>278</v>
       </c>
@@ -5620,13 +5620,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Feuil5"/>
   <dimension ref="A1:C169"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>167</v>
       </c>
@@ -5637,7 +5637,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>pi</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -5673,7 +5673,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -5685,7 +5685,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -5709,7 +5709,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -5745,7 +5745,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -5769,7 +5769,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>86</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -5805,7 +5805,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -5829,7 +5829,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -5841,7 +5841,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -5853,7 +5853,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -5865,7 +5865,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -5889,7 +5889,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -5901,7 +5901,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -5913,7 +5913,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -5925,7 +5925,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -5937,7 +5937,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -5949,7 +5949,7 @@
         <v>root_growth_T_ref</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -5961,7 +5961,7 @@
         <v>root_growth_A</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -5973,7 +5973,7 @@
         <v>root_growth_B</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>95</v>
       </c>
@@ -5985,7 +5985,7 @@
         <v>root_growth_C</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>96</v>
       </c>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>97</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>98</v>
       </c>
@@ -6021,7 +6021,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>99</v>
       </c>
@@ -6033,7 +6033,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>100</v>
       </c>
@@ -6045,7 +6045,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>61</v>
       </c>
@@ -6057,7 +6057,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -6069,7 +6069,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>101</v>
       </c>
@@ -6081,7 +6081,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>102</v>
       </c>
@@ -6093,7 +6093,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>103</v>
       </c>
@@ -6105,7 +6105,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -6117,7 +6117,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>76</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>105</v>
       </c>
@@ -6141,7 +6141,7 @@
         <v>expected_C_sucrose_root</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>106</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>expected_C_hexose_root</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>107</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>expected_C_hexose_soil</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>108</v>
       </c>
@@ -6177,7 +6177,7 @@
         <v>expected_C_hexose_reserve</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>65</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>77</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -6213,7 +6213,7 @@
         <v>surfacic_unloading_rate_reference</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>110</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>surfacic_unloading_rate_primordium</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -6237,7 +6237,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>111</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>112</v>
       </c>
@@ -6261,7 +6261,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>113</v>
       </c>
@@ -6273,7 +6273,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>114</v>
       </c>
@@ -6285,7 +6285,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -6297,7 +6297,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>115</v>
       </c>
@@ -6309,7 +6309,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>116</v>
       </c>
@@ -6321,7 +6321,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>117</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>118</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -6369,7 +6369,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -6381,7 +6381,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>56</v>
       </c>
@@ -6405,7 +6405,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>58</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -6429,7 +6429,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>119</v>
       </c>
@@ -6441,7 +6441,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>120</v>
       </c>
@@ -6453,7 +6453,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>121</v>
       </c>
@@ -6465,7 +6465,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>122</v>
       </c>
@@ -6477,7 +6477,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -6501,7 +6501,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>123</v>
       </c>
@@ -6513,7 +6513,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>124</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>125</v>
       </c>
@@ -6537,7 +6537,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>126</v>
       </c>
@@ -6549,7 +6549,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>74</v>
       </c>
@@ -6561,7 +6561,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>127</v>
       </c>
@@ -6573,7 +6573,7 @@
         <v>expected_exudation_efflux</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>128</v>
       </c>
@@ -6597,7 +6597,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>129</v>
       </c>
@@ -6609,7 +6609,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>130</v>
       </c>
@@ -6621,7 +6621,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>131</v>
       </c>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -6645,7 +6645,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>80</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>132</v>
       </c>
@@ -6669,7 +6669,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>133</v>
       </c>
@@ -6681,7 +6681,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>134</v>
       </c>
@@ -6693,7 +6693,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>135</v>
       </c>
@@ -6705,7 +6705,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -6717,7 +6717,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>136</v>
       </c>
@@ -6729,7 +6729,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>137</v>
       </c>
@@ -6741,7 +6741,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>138</v>
       </c>
@@ -6753,7 +6753,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>139</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>140</v>
       </c>
@@ -6777,7 +6777,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>141</v>
       </c>
@@ -6789,7 +6789,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>142</v>
       </c>
@@ -6801,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>143</v>
       </c>
@@ -6813,7 +6813,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>144</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>145</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>146</v>
       </c>
@@ -6849,7 +6849,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>147</v>
       </c>
@@ -6861,7 +6861,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>148</v>
       </c>
@@ -6873,7 +6873,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>149</v>
       </c>
@@ -6885,7 +6885,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>150</v>
       </c>
@@ -6897,7 +6897,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>151</v>
       </c>
@@ -6909,7 +6909,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>152</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>153</v>
       </c>
@@ -6933,7 +6933,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>154</v>
       </c>
@@ -6945,7 +6945,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>155</v>
       </c>
@@ -6957,7 +6957,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>156</v>
       </c>
@@ -6969,7 +6969,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>157</v>
       </c>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>158</v>
       </c>
@@ -6993,7 +6993,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>159</v>
       </c>
@@ -7005,7 +7005,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>160</v>
       </c>
@@ -7017,7 +7017,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>161</v>
       </c>
@@ -7029,7 +7029,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>162</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>163</v>
       </c>
@@ -7053,7 +7053,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>164</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>165</v>
       </c>
@@ -7077,7 +7077,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>166</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>59</v>
       </c>
@@ -7101,7 +7101,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>62</v>
       </c>
@@ -7113,7 +7113,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>64</v>
       </c>
@@ -7125,7 +7125,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>63</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>82</v>
       </c>
@@ -7149,7 +7149,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>83</v>
       </c>
@@ -7161,7 +7161,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>85</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>84</v>
       </c>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>2</v>
       </c>
@@ -7197,7 +7197,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -7209,7 +7209,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -7221,7 +7221,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>20</v>
       </c>
@@ -7233,7 +7233,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>0</v>
       </c>
@@ -7245,7 +7245,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>1</v>
       </c>
@@ -7257,7 +7257,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>6</v>
       </c>
@@ -7269,7 +7269,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>7</v>
       </c>
@@ -7281,7 +7281,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -7293,7 +7293,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -7305,7 +7305,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>10</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>11</v>
       </c>
@@ -7329,7 +7329,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>12</v>
       </c>
@@ -7341,7 +7341,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -7353,7 +7353,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -7365,7 +7365,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>15</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>17</v>
       </c>
@@ -7401,7 +7401,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -7413,7 +7413,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>19</v>
       </c>
@@ -7425,7 +7425,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -7437,7 +7437,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>22</v>
       </c>
@@ -7449,7 +7449,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>23</v>
       </c>
@@ -7461,7 +7461,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -7473,7 +7473,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>25</v>
       </c>
@@ -7485,7 +7485,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -7497,7 +7497,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>27</v>
       </c>
@@ -7509,7 +7509,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>28</v>
       </c>
@@ -7518,7 +7518,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>29</v>
       </c>
@@ -7527,7 +7527,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -7536,7 +7536,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>31</v>
       </c>
@@ -7545,7 +7545,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -7554,7 +7554,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>33</v>
       </c>
@@ -7563,7 +7563,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -7572,7 +7572,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>35</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>36</v>
       </c>
@@ -7590,7 +7590,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>37</v>
       </c>
@@ -7599,7 +7599,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>38</v>
       </c>
@@ -7608,7 +7608,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>170</v>
       </c>

</xml_diff>

<commit_message>
diagnosed AA deficits (lack of polarization of unloading)
</commit_message>
<xml_diff>
--- a/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
+++ b/simulations/inputs/outputs_validation_root_cynaps_V0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp46580\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp25823\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828CF325-9EA2-4EB3-97CC-8ABFC52BD208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCA5BA5-B128-42BB-AFFB-19DEB326D58C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="341">
   <si>
     <t>input_file</t>
   </si>
@@ -1055,9 +1055,6 @@
     <t>Prefered validating on Cao since it is field conditions matching Swinnen temperatures</t>
   </si>
   <si>
-    <t>Seems odd to restrict that low, check further references</t>
-  </si>
-  <si>
     <t>deficit_Nm</t>
   </si>
   <si>
@@ -1086,6 +1083,12 @@
   </si>
   <si>
     <t>deficit_xylem_Nm</t>
+  </si>
+  <si>
+    <t>Devienne et al. 1994</t>
+  </si>
+  <si>
+    <t>Azevedo et al. 2009</t>
   </si>
 </sst>
 </file>
@@ -3363,7 +3366,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3510,7 +3513,7 @@
         <v>171</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>314</v>
+        <v>340</v>
       </c>
       <c r="F3" s="4" t="e">
         <f>NA()</f>
@@ -3524,20 +3527,16 @@
         <f t="array" ref="H3">IFERROR(SQRT(AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!W:W, 'reference_list&amp;conversion'!$A:$A=$B3)^2) + _xlfn.VAR.S(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B3)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))),NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I3" s="9" cm="1">
-        <f t="array" ref="I3">MIN(_xlfn._xlws.FILTER('reference_list&amp;conversion'!X:X,('reference_list&amp;conversion'!$A:$A=$B3)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>7.3095238095238015E-5</v>
-      </c>
-      <c r="J3" s="9" cm="1">
-        <f t="array" ref="J3">MAX(_xlfn._xlws.FILTER('reference_list&amp;conversion'!Y:Y,('reference_list&amp;conversion'!$A:$A=$B3)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>2.4724089635854265E-4</v>
+      <c r="I3" s="9">
+        <v>6.3949999999999999E-4</v>
+      </c>
+      <c r="J3" s="9">
+        <v>1.186E-3</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>329</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="L3" s="9"/>
       <c r="M3" s="9" t="s">
         <v>188</v>
       </c>
@@ -3676,37 +3675,39 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>193</v>
+        <v>339</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>185</v>
       </c>
       <c r="G6" s="9">
-        <v>8.7999999999999998E-5</v>
+        <v>5.4999999999999996E-9</v>
       </c>
       <c r="H6" s="9" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
       <c r="I6" s="9">
-        <v>1.0000000000000001E-5</v>
+        <f>0.6*0.000001*10/3600</f>
+        <v>1.6666666666666667E-9</v>
       </c>
       <c r="J6" s="9">
-        <v>4.6999999999999999E-4</v>
-      </c>
-      <c r="K6" s="4" t="s">
+        <f>8.2*0.000001*10/3600</f>
+        <v>2.2777777777777775E-8</v>
+      </c>
+      <c r="K6" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="L6" s="4"/>
+      <c r="L6" s="9"/>
       <c r="M6" s="4" t="s">
         <v>187</v>
       </c>
@@ -3733,13 +3734,13 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>239</v>
+        <v>195</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>241</v>
+        <v>196</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>193</v>
@@ -3748,7 +3749,7 @@
         <v>185</v>
       </c>
       <c r="G7" s="9">
-        <v>1E-8</v>
+        <v>8.7999999999999998E-5</v>
       </c>
       <c r="H7" s="9" t="e">
         <f>NA()</f>
@@ -3758,7 +3759,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="J7" s="9">
-        <v>6.9999999999999999E-4</v>
+        <v>4.6999999999999999E-4</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>175</v>
@@ -3790,33 +3791,32 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>326</v>
+        <v>239</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>243</v>
+        <v>192</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="F8" s="4" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G8" s="4">
-        <v>0</v>
+        <v>193</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="G8" s="9">
+        <v>1E-8</v>
       </c>
       <c r="H8" s="9" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
       <c r="I8" s="9">
-        <v>-10000000</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="J8" s="9">
-        <v>-100</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>175</v>
@@ -3831,11 +3831,11 @@
       <c r="O8" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="P8" s="4" t="s">
+      <c r="P8" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q8" s="4" t="s">
         <v>179</v>
-      </c>
-      <c r="Q8" s="15" t="s">
-        <v>175</v>
       </c>
       <c r="R8" s="4" t="e">
         <f>NA()</f>
@@ -3848,32 +3848,33 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>240</v>
+        <v>326</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>192</v>
+        <v>243</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="G9" s="9">
-        <v>1E-4</v>
+        <v>250</v>
+      </c>
+      <c r="F9" s="4" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
       </c>
       <c r="H9" s="9" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
       <c r="I9" s="9">
-        <v>1.0000000000000001E-5</v>
+        <v>-10000000</v>
       </c>
       <c r="J9" s="9">
-        <v>6.9999999999999999E-4</v>
+        <v>-100</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>175</v>
@@ -3885,14 +3886,14 @@
       <c r="N9" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="O9" s="15" t="s">
-        <v>175</v>
+      <c r="O9" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="Q9" s="4" t="s">
-        <v>179</v>
+      <c r="Q9" s="15" t="s">
+        <v>175</v>
       </c>
       <c r="R9" s="4" t="e">
         <f>NA()</f>
@@ -3905,51 +3906,48 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>304</v>
+        <v>242</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>192</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>251</v>
+        <v>193</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="G10" s="4" cm="1">
-        <f t="array" ref="G10">AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B10)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>9.046003613776749E-10</v>
-      </c>
-      <c r="H10" s="4" cm="1">
-        <f t="array" ref="H10">IFERROR(SQRT(AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!W:W, 'reference_list&amp;conversion'!$A:$A=$B10)^2) + _xlfn.VAR.S(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B10)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))),NA())</f>
-        <v>1.2809900539560876E-9</v>
-      </c>
-      <c r="I10" s="4" cm="1">
-        <f t="array" ref="I10">MIN(_xlfn._xlws.FILTER('reference_list&amp;conversion'!X:X,('reference_list&amp;conversion'!$A:$A=$B10)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>8.3333333333333338E-13</v>
-      </c>
-      <c r="J10" s="4" cm="1">
-        <f t="array" ref="J10">MAX(_xlfn._xlws.FILTER('reference_list&amp;conversion'!Y:Y,('reference_list&amp;conversion'!$A:$A=$B10)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>2.0663913021965896E-9</v>
+      <c r="G10" s="9">
+        <v>1E-4</v>
+      </c>
+      <c r="H10" s="9" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I10" s="9">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J10" s="9">
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>175</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N10" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="O10" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="P10" s="4" t="s">
         <v>179</v>
-      </c>
-      <c r="P10" s="15" t="s">
-        <v>175</v>
       </c>
       <c r="Q10" s="4" t="s">
         <v>179</v>
@@ -3965,44 +3963,42 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>293</v>
+        <v>248</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>249</v>
+        <v>304</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>192</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>294</v>
+        <v>251</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>185</v>
       </c>
       <c r="G11" s="4" cm="1">
         <f t="array" ref="G11">AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B11)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>6.9313417190775683E-9</v>
-      </c>
-      <c r="H11" s="4" t="e" cm="1">
+        <v>9.046003613776749E-10</v>
+      </c>
+      <c r="H11" s="4" cm="1">
         <f t="array" ref="H11">IFERROR(SQRT(AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!W:W, 'reference_list&amp;conversion'!$A:$A=$B11)^2) + _xlfn.VAR.S(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B11)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))),NA())</f>
-        <v>#N/A</v>
+        <v>1.2809900539560876E-9</v>
       </c>
       <c r="I11" s="4" cm="1">
         <f t="array" ref="I11">MIN(_xlfn._xlws.FILTER('reference_list&amp;conversion'!X:X,('reference_list&amp;conversion'!$A:$A=$B11)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>2.8432914046121594E-9</v>
+        <v>8.3333333333333338E-13</v>
       </c>
       <c r="J11" s="4" cm="1">
         <f t="array" ref="J11">MAX(_xlfn._xlws.FILTER('reference_list&amp;conversion'!Y:Y,('reference_list&amp;conversion'!$A:$A=$B11)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
-        <v>1.101939203354298E-8</v>
+        <v>2.0663913021965896E-9</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>328</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N11" s="4" t="s">
         <v>179</v>
@@ -4027,39 +4023,44 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>339</v>
+        <v>293</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>331</v>
+        <v>192</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="F12" s="4" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G12" s="4">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4">
-        <v>0</v>
+        <v>294</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="G12" s="4" cm="1">
+        <f t="array" ref="G12">AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B12)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
+        <v>6.9313417190775683E-9</v>
+      </c>
+      <c r="H12" s="4" t="e" cm="1">
+        <f t="array" ref="H12">IFERROR(SQRT(AVERAGE(_xlfn._xlws.FILTER('reference_list&amp;conversion'!W:W, 'reference_list&amp;conversion'!$A:$A=$B12)^2) + _xlfn.VAR.S(_xlfn._xlws.FILTER('reference_list&amp;conversion'!V:V, ('reference_list&amp;conversion'!$A:$A=$B12)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I12" s="4" cm="1">
+        <f t="array" ref="I12">MIN(_xlfn._xlws.FILTER('reference_list&amp;conversion'!X:X,('reference_list&amp;conversion'!$A:$A=$B12)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
+        <v>2.8432914046121594E-9</v>
+      </c>
+      <c r="J12" s="4" cm="1">
+        <f t="array" ref="J12">MAX(_xlfn._xlws.FILTER('reference_list&amp;conversion'!Y:Y,('reference_list&amp;conversion'!$A:$A=$B12)*IF($A$3="no",1,'reference_list&amp;conversion'!$D:$D=$A$3)))</f>
+        <v>1.101939203354298E-8</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="L12" s="4"/>
+        <v>179</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>328</v>
+      </c>
       <c r="M12" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N12" s="4" t="s">
         <v>179</v>
@@ -4084,13 +4085,13 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>330</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>331</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>250</v>
@@ -4141,13 +4142,13 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>250</v>
@@ -4198,13 +4199,13 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>250</v>
@@ -4255,13 +4256,13 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>250</v>
@@ -4312,13 +4313,13 @@
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>250</v>
@@ -4369,13 +4370,13 @@
     </row>
     <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>250</v>
@@ -4426,13 +4427,13 @@
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>250</v>
@@ -4481,11 +4482,64 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="Q30" s="10"/>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="F20" s="4" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="P20" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q20" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="R20" s="4" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="Q31" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K12:K19">
+  <conditionalFormatting sqref="K13:K20">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -4502,8 +4556,8 @@
       <formula>"FALSE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L11">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="L13:L20">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4514,8 +4568,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12:L19">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="K2:L12">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>